<commit_message>
Standardize suite sample fields across all DataLund visuals
Align Excel columns and help copy to the shared field wells people
already use (Start Date, End Date, Progress 0–100, Group, Resource),
add How-to sheets on every sample, and document the contract on Support.

Co-authored-by: JonasL <Prez0@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/public/downloads/DatalundSuiteSample.xlsx
+++ b/public/downloads/DatalundSuiteSample.xlsx
@@ -431,7 +431,7 @@
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
     <col width="18" customWidth="1" min="9" max="9"/>
     <col width="26" customWidth="1" min="10" max="10"/>
@@ -450,7 +450,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Phase</t>
+          <t>Group</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -465,12 +465,12 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Start date</t>
+          <t>Start Date</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Estimated end</t>
+          <t>End Date</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
@@ -866,12 +866,12 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Start</t>
+          <t>Start Date</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>End</t>
+          <t>End Date</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -918,7 +918,7 @@
         <v>46198</v>
       </c>
       <c r="E2" t="n">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -954,7 +954,7 @@
         <v>46208</v>
       </c>
       <c r="E3" t="n">
-        <v>0.9</v>
+        <v>90</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -990,7 +990,7 @@
         <v>46223</v>
       </c>
       <c r="E4" t="n">
-        <v>0.75</v>
+        <v>75</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -1026,7 +1026,7 @@
         <v>46270</v>
       </c>
       <c r="E5" t="n">
-        <v>0.2</v>
+        <v>20</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -1062,7 +1062,7 @@
         <v>46188</v>
       </c>
       <c r="E6" t="n">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -1098,7 +1098,7 @@
         <v>46254</v>
       </c>
       <c r="E7" t="n">
-        <v>0.4</v>
+        <v>40</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -1170,7 +1170,7 @@
         <v>46228</v>
       </c>
       <c r="E9" t="n">
-        <v>0.5</v>
+        <v>50</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
@@ -1206,7 +1206,7 @@
         <v>46239</v>
       </c>
       <c r="E10" t="n">
-        <v>0.15</v>
+        <v>15</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -1278,7 +1278,7 @@
         <v>46203</v>
       </c>
       <c r="E12" t="n">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -1314,7 +1314,7 @@
         <v>46244</v>
       </c>
       <c r="E13" t="n">
-        <v>0.85</v>
+        <v>85</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
@@ -1350,7 +1350,7 @@
         <v>46259</v>
       </c>
       <c r="E14" t="n">
-        <v>0.3</v>
+        <v>30</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
@@ -1386,7 +1386,7 @@
         <v>46234</v>
       </c>
       <c r="E15" t="n">
-        <v>0.7</v>
+        <v>70</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
@@ -1422,7 +1422,7 @@
         <v>46249</v>
       </c>
       <c r="E16" t="n">
-        <v>0.25</v>
+        <v>25</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
@@ -1458,7 +1458,7 @@
         <v>46296</v>
       </c>
       <c r="E17" t="n">
-        <v>0.1</v>
+        <v>10</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
@@ -1494,7 +1494,7 @@
         <v>46280</v>
       </c>
       <c r="E18" t="n">
-        <v>0.05</v>
+        <v>5</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
@@ -1530,7 +1530,7 @@
         <v>46234</v>
       </c>
       <c r="E19" t="n">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -1566,7 +1566,7 @@
         <v>46249</v>
       </c>
       <c r="E20" t="n">
-        <v>0.55</v>
+        <v>55</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
@@ -1602,7 +1602,7 @@
         <v>46296</v>
       </c>
       <c r="E21" t="n">
-        <v>0.15</v>
+        <v>15</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
@@ -1638,7 +1638,7 @@
         <v>14</v>
       </c>
       <c r="E22" t="n">
-        <v>0.1</v>
+        <v>10</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
@@ -1710,7 +1710,7 @@
         <v>46266</v>
       </c>
       <c r="E24" t="n">
-        <v>0.15</v>
+        <v>15</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
@@ -1744,7 +1744,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A21"/>
+  <dimension ref="A1:A27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="90" customWidth="1" min="1" max="1"/>
@@ -1753,7 +1753,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Datalund suite sample — one workbook for Gantt, Resource Load, and Task List</t>
+          <t>DataLund suite sample — one workbook for Gantt, Resource Load, and Task List</t>
         </is>
       </c>
     </row>
@@ -1763,52 +1763,52 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1. Power BI Desktop → Get data → Excel workbook → this file.</t>
+          <t>Shared field wells (same names across the suite)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2. Load both Projects and Tasks. Relate Tasks[Project] → Projects[Project] (many-to-one).</t>
+          <t xml:space="preserve">  Task / Project · Start Date · End Date · Duration · Progress · Group · Resource / Project lead · RAG · Tooltips</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>3. Import each .pbiviz (Visualizations … → Import a visual from a file).</t>
+          <t xml:space="preserve">  Progress is 0–100 here (visuals also accept 0–1). RAG: Red / Amber / Green (also Rød / Gul / Grønn).</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr"/>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  End Date or Duration is enough for timeline bars.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>DataLund Task List (Projects sheet)</t>
-        </is>
-      </c>
+      <c r="A7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Project → Project | RAG → RAG | Group → Phase | Project lead → Project lead</t>
+          <t>1. Power BI Desktop → Get data → Excel workbook → this file.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Progress → Progress | Start Date → Start date | End Date → Estimated end</t>
+          <t>2. Load both Projects and Tasks. Relate Tasks[Project] → Projects[Project] (many-to-one).</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Tooltips → Next milestone, Obstacles, Notes</t>
+          <t>3. Import each .pbiviz (Visualizations … → Import a visual from a file).</t>
         </is>
       </c>
     </row>
@@ -1818,62 +1818,100 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>DataLund Gantt chart (Tasks sheet)</t>
+          <t>DataLund Task List (Projects sheet)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Task → Task | Start Date → Start | End Date → End | Duration → Duration</t>
+          <t xml:space="preserve">  Project → Project | RAG → RAG | Group → Group | Project lead → Project lead</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Progress → Progress | Group → Group | Resource → Resource</t>
+          <t xml:space="preserve">  Progress → Progress | Start Date → Start Date | End Date → End Date</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr"/>
+      <c r="A15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Tooltips → Next milestone, Obstacles, Notes</t>
+        </is>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>DataLund Resource Load (Tasks sheet)</t>
-        </is>
-      </c>
+      <c r="A16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Resource → Resource | Task → Task | Start Date → Start | End Date → End</t>
+          <t>DataLund Gantt chart (Tasks sheet)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Progress → Progress | Group → Group</t>
+          <t xml:space="preserve">  Task → Task | Start Date → Start Date | End Date → End Date | Duration → Duration</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr"/>
+      <c r="A19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Progress → Progress | Group → Group | Resource → Resource</t>
+        </is>
+      </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Tip: put Task List on the page and cross-filter Gantt + Resource Load from selected projects.</t>
-        </is>
-      </c>
+      <c r="A20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Scope freeze is a zero-duration milestone. QA soak uses Duration instead of End.</t>
+          <t>DataLund Resource Load (Tasks sheet)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Resource → Resource | Task → Task | Start Date → Start Date | End Date → End Date | Duration → Duration</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Progress → Progress | Group → Group</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Tip: put RAG on Tooltips if you want status on hover.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Tip: put Task List on the page and cross-filter Gantt + Resource Load from selected projects.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Scope freeze is a zero-duration milestone. QA soak uses Duration instead of End Date.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Strip starter Excels to columns PMs actually maintain
Drop Duration, Tooltips, and task-level RAG from samples; keep seven
core project/task fields, fewer rows, and shorter Start here copy so
the starter model converts instead of overwhelming.

Co-authored-by: JonasL <Prez0@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/public/downloads/DatalundSuiteSample.xlsx
+++ b/public/downloads/DatalundSuiteSample.xlsx
@@ -12,8 +12,8 @@
     <sheet name="Tasks" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Projects'!$A$1:$J$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Tasks'!$A$1:$I$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Projects'!$A$1:$G$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Tasks'!$A$1:$G$13</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -559,15 +559,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F32"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="92" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="88" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="36" customHeight="1">
@@ -580,21 +579,19 @@
       <c r="C1" s="2" t="n"/>
       <c r="D1" s="2" t="n"/>
       <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
     </row>
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>A simple starter workbook for Task List, Gantt, and Resource Load</t>
+          <t>Seven columns. Replace the rows with your projects and tasks.</t>
         </is>
       </c>
       <c r="B2" s="4" t="n"/>
       <c r="C2" s="4" t="n"/>
       <c r="D2" s="4" t="n"/>
       <c r="E2" s="4" t="n"/>
-      <c r="F2" s="4" t="n"/>
-    </row>
-    <row r="4" ht="22" customHeight="1">
+    </row>
+    <row r="4" ht="20" customHeight="1">
       <c r="A4" s="5" t="inlineStr">
         <is>
           <t>Quick start</t>
@@ -604,158 +601,78 @@
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>1. Import the visuals</t>
+          <t>1. Import the three .pbiviz files from datalund.no</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="inlineStr">
-        <is>
-          <t>Download the suite zip from datalund.no, then in Power BI Desktop:</t>
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>2. Load Projects and Tasks — relate Tasks[Project] → Projects[Project]</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="inlineStr">
-        <is>
-          <t>Visualizations … → Import a visual from a file → pick each .pbiviz.</t>
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>3. Bind matching column names (see below)</t>
         </is>
       </c>
     </row>
     <row r="8"/>
-    <row r="9">
-      <c r="A9" s="6" t="inlineStr">
-        <is>
-          <t>2. Load this workbook</t>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>What to maintain</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>Home → Get data → Excel workbook → load Projects and Tasks.</t>
+          <t>Projects → DataLund Task List: Project, RAG, Group, Project lead, Progress, Start Date, End Date</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>Relate Tasks[Project] → Projects[Project] (many-to-one).</t>
-        </is>
-      </c>
-    </row>
-    <row r="12"/>
+          <t>Tasks → Gantt + Resource Load: Task, Start Date, End Date, Progress, Group, Resource, Project</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>Progress is 0–100. RAG is Red / Amber / Green (or Rød / Gul / Grønn).</t>
+        </is>
+      </c>
+    </row>
     <row r="13">
-      <c r="A13" s="6" t="inlineStr">
-        <is>
-          <t>3. Bind the same columns everywhere</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="7" t="inlineStr">
-        <is>
-          <t>Minimum for Task List: Project (+ RAG and Progress look great).</t>
-        </is>
-      </c>
-    </row>
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>Same start and end date = milestone. Duration and Tooltips are optional later — not in this starter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14"/>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>Minimum for Gantt / Resource Load: Task, Start Date, and End Date or Duration.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="7" t="inlineStr">
-        <is>
-          <t>Then add Progress, Group, and Resource / Project lead.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17"/>
+          <t>Put Task List on the page, click a project — Gantt and Resource Load follow.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16"/>
+    <row r="17">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>https://datalund.no</t>
+        </is>
+      </c>
+    </row>
     <row r="18">
-      <c r="A18" s="6" t="inlineStr">
-        <is>
-          <t>4. Build one page</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="7" t="inlineStr">
-        <is>
-          <t>Put Task List on the left. Click a project — Gantt and Resource Load follow.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20"/>
-    <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="5" t="inlineStr">
-        <is>
-          <t>What’s in the sheets</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="7" t="inlineStr">
-        <is>
-          <t>Projects — portfolio rows for DataLund Task List (Lists-style names).</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="7" t="inlineStr">
-        <is>
-          <t>Tasks — assignment rows for DataLund Gantt and Resource Load.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="8" t="inlineStr">
-        <is>
-          <t>Progress is 0–100. RAG is Red / Amber / Green (also Rød / Gul / Grønn).</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="8" t="inlineStr">
-        <is>
-          <t>Scope freeze is a milestone (same start and end). QA soak uses Duration instead of End Date.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26"/>
-    <row r="27" ht="20" customHeight="1">
-      <c r="A27" s="5" t="inlineStr">
-        <is>
-          <t>Make it yours</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="7" t="inlineStr">
-        <is>
-          <t>Replace the sample rows with your projects and tasks. Keep the column headers.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="7" t="inlineStr">
-        <is>
-          <t>Same field names work across the whole DataLund suite.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30"/>
-    <row r="31">
-      <c r="A31" s="9" t="inlineStr">
-        <is>
-          <t>https://datalund.no</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="8" t="inlineStr">
+      <c r="A18" s="8" t="inlineStr">
         <is>
           <t>Free Power BI visuals · support@datalund.no</t>
         </is>
@@ -763,11 +680,11 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A1:E1"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A31" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A17" r:id="rId1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -780,7 +697,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -790,9 +707,6 @@
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="28" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
@@ -831,21 +745,6 @@
           <t>End Date</t>
         </is>
       </c>
-      <c r="H1" s="10" t="inlineStr">
-        <is>
-          <t>Next milestone</t>
-        </is>
-      </c>
-      <c r="I1" s="10" t="inlineStr">
-        <is>
-          <t>Obstacles</t>
-        </is>
-      </c>
-      <c r="J1" s="10" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="11" t="inlineStr">
@@ -877,17 +776,6 @@
       <c r="G2" s="14" t="n">
         <v>46284</v>
       </c>
-      <c r="H2" s="11" t="inlineStr">
-        <is>
-          <t>FAT complete</t>
-        </is>
-      </c>
-      <c r="I2" s="11" t="inlineStr"/>
-      <c r="J2" s="11" t="inlineStr">
-        <is>
-          <t>On track for Q3</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" s="15" t="inlineStr">
@@ -919,21 +807,6 @@
       <c r="G3" s="18" t="n">
         <v>46264</v>
       </c>
-      <c r="H3" s="15" t="inlineStr">
-        <is>
-          <t>Cable pull</t>
-        </is>
-      </c>
-      <c r="I3" s="15" t="inlineStr">
-        <is>
-          <t>Weather window</t>
-        </is>
-      </c>
-      <c r="J3" s="15" t="inlineStr">
-        <is>
-          <t>Watch supplier lead time</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
@@ -965,21 +838,6 @@
       <c r="G4" s="14" t="n">
         <v>46254</v>
       </c>
-      <c r="H4" s="11" t="inlineStr">
-        <is>
-          <t>Scope freeze</t>
-        </is>
-      </c>
-      <c r="I4" s="11" t="inlineStr">
-        <is>
-          <t>Budget overrun</t>
-        </is>
-      </c>
-      <c r="J4" s="11" t="inlineStr">
-        <is>
-          <t>Critical path slip</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" s="15" t="inlineStr">
@@ -1011,17 +869,6 @@
       <c r="G5" s="18" t="n">
         <v>46259</v>
       </c>
-      <c r="H5" s="15" t="inlineStr">
-        <is>
-          <t>UAT</t>
-        </is>
-      </c>
-      <c r="I5" s="15" t="inlineStr"/>
-      <c r="J5" s="15" t="inlineStr">
-        <is>
-          <t>Near release</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" s="11" t="inlineStr">
@@ -1053,20 +900,9 @@
       <c r="G6" s="14" t="n">
         <v>46424</v>
       </c>
-      <c r="H6" s="11" t="inlineStr">
-        <is>
-          <t>Permits</t>
-        </is>
-      </c>
-      <c r="I6" s="11" t="inlineStr"/>
-      <c r="J6" s="11" t="inlineStr">
-        <is>
-          <t>Replace these rows with your projects</t>
-        </is>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J6"/>
+  <autoFilter ref="A1:G6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1078,18 +914,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I18"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
@@ -1110,32 +944,22 @@
       </c>
       <c r="D1" s="10" t="inlineStr">
         <is>
-          <t>Duration</t>
+          <t>Progress</t>
         </is>
       </c>
       <c r="E1" s="10" t="inlineStr">
         <is>
-          <t>Progress</t>
+          <t>Group</t>
         </is>
       </c>
       <c r="F1" s="10" t="inlineStr">
         <is>
-          <t>Group</t>
+          <t>Resource</t>
         </is>
       </c>
       <c r="G1" s="10" t="inlineStr">
         <is>
-          <t>Resource</t>
-        </is>
-      </c>
-      <c r="H1" s="10" t="inlineStr">
-        <is>
           <t>Project</t>
-        </is>
-      </c>
-      <c r="I1" s="10" t="inlineStr">
-        <is>
-          <t>RAG</t>
         </is>
       </c>
     </row>
@@ -1151,625 +975,368 @@
       <c r="C2" s="14" t="n">
         <v>46198</v>
       </c>
-      <c r="D2" s="11" t="n"/>
-      <c r="E2" s="13" t="n">
+      <c r="D2" s="13" t="n">
         <v>100</v>
       </c>
+      <c r="E2" s="11" t="inlineStr">
+        <is>
+          <t>Delivery</t>
+        </is>
+      </c>
       <c r="F2" s="11" t="inlineStr">
         <is>
-          <t>Delivery</t>
+          <t>Ada Ng</t>
         </is>
       </c>
       <c r="G2" s="11" t="inlineStr">
         <is>
-          <t>Ada Ng</t>
-        </is>
-      </c>
-      <c r="H2" s="11" t="inlineStr">
-        <is>
           <t>North Sea Hub</t>
-        </is>
-      </c>
-      <c r="I2" s="12" t="inlineStr">
-        <is>
-          <t>Green</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="15" t="inlineStr">
         <is>
-          <t>Wireframes</t>
+          <t>API design</t>
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>46193</v>
+        <v>46204</v>
       </c>
       <c r="C3" s="18" t="n">
-        <v>46208</v>
-      </c>
-      <c r="D3" s="15" t="n"/>
-      <c r="E3" s="17" t="n">
-        <v>90</v>
+        <v>46223</v>
+      </c>
+      <c r="D3" s="17" t="n">
+        <v>75</v>
+      </c>
+      <c r="E3" s="15" t="inlineStr">
+        <is>
+          <t>Delivery</t>
+        </is>
       </c>
       <c r="F3" s="15" t="inlineStr">
         <is>
-          <t>Delivery</t>
+          <t>Sam Ortiz</t>
         </is>
       </c>
       <c r="G3" s="15" t="inlineStr">
         <is>
-          <t>Jordan Lee</t>
-        </is>
-      </c>
-      <c r="H3" s="15" t="inlineStr">
-        <is>
           <t>North Sea Hub</t>
-        </is>
-      </c>
-      <c r="I3" s="12" t="inlineStr">
-        <is>
-          <t>Green</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>API design</t>
+          <t>FAT prep</t>
         </is>
       </c>
       <c r="B4" s="14" t="n">
-        <v>46204</v>
+        <v>46254</v>
       </c>
       <c r="C4" s="14" t="n">
-        <v>46223</v>
-      </c>
-      <c r="D4" s="11" t="n"/>
-      <c r="E4" s="13" t="n">
-        <v>75</v>
+        <v>46270</v>
+      </c>
+      <c r="D4" s="13" t="n">
+        <v>20</v>
+      </c>
+      <c r="E4" s="11" t="inlineStr">
+        <is>
+          <t>Delivery</t>
+        </is>
       </c>
       <c r="F4" s="11" t="inlineStr">
         <is>
-          <t>Delivery</t>
+          <t>Ada Ng</t>
         </is>
       </c>
       <c r="G4" s="11" t="inlineStr">
         <is>
-          <t>Sam Ortiz</t>
-        </is>
-      </c>
-      <c r="H4" s="11" t="inlineStr">
-        <is>
           <t>North Sea Hub</t>
-        </is>
-      </c>
-      <c r="I4" s="12" t="inlineStr">
-        <is>
-          <t>Green</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="15" t="inlineStr">
         <is>
-          <t>FAT prep</t>
+          <t>Cable pull</t>
         </is>
       </c>
       <c r="B5" s="18" t="n">
+        <v>46204</v>
+      </c>
+      <c r="C5" s="18" t="n">
         <v>46254</v>
       </c>
-      <c r="C5" s="18" t="n">
-        <v>46270</v>
-      </c>
-      <c r="D5" s="15" t="n"/>
-      <c r="E5" s="17" t="n">
-        <v>20</v>
+      <c r="D5" s="17" t="n">
+        <v>40</v>
+      </c>
+      <c r="E5" s="15" t="inlineStr">
+        <is>
+          <t>Delivery</t>
+        </is>
       </c>
       <c r="F5" s="15" t="inlineStr">
         <is>
-          <t>Delivery</t>
+          <t>Bo Berg</t>
         </is>
       </c>
       <c r="G5" s="15" t="inlineStr">
         <is>
-          <t>Ada Ng</t>
-        </is>
-      </c>
-      <c r="H5" s="15" t="inlineStr">
-        <is>
-          <t>North Sea Hub</t>
-        </is>
-      </c>
-      <c r="I5" s="16" t="inlineStr">
-        <is>
-          <t>Amber</t>
+          <t>Arctic Link</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="11" t="inlineStr">
         <is>
-          <t>Cable survey</t>
+          <t>Weather hold</t>
         </is>
       </c>
       <c r="B6" s="14" t="n">
-        <v>46154</v>
+        <v>46244</v>
       </c>
       <c r="C6" s="14" t="n">
-        <v>46188</v>
-      </c>
-      <c r="D6" s="11" t="n"/>
-      <c r="E6" s="13" t="n">
-        <v>100</v>
+        <v>46252</v>
+      </c>
+      <c r="D6" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="11" t="inlineStr">
+        <is>
+          <t>Delivery</t>
+        </is>
       </c>
       <c r="F6" s="11" t="inlineStr">
         <is>
-          <t>Delivery</t>
+          <t>Riley Chen</t>
         </is>
       </c>
       <c r="G6" s="11" t="inlineStr">
         <is>
-          <t>Bo Berg</t>
-        </is>
-      </c>
-      <c r="H6" s="11" t="inlineStr">
-        <is>
           <t>Arctic Link</t>
-        </is>
-      </c>
-      <c r="I6" s="12" t="inlineStr">
-        <is>
-          <t>Green</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="15" t="inlineStr">
         <is>
-          <t>Cable pull</t>
+          <t>On-call week</t>
         </is>
       </c>
       <c r="B7" s="18" t="n">
-        <v>46204</v>
+        <v>46252</v>
       </c>
       <c r="C7" s="18" t="n">
-        <v>46254</v>
-      </c>
-      <c r="D7" s="15" t="n"/>
-      <c r="E7" s="17" t="n">
-        <v>40</v>
+        <v>46258</v>
+      </c>
+      <c r="D7" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="15" t="inlineStr">
+        <is>
+          <t>Delivery</t>
+        </is>
       </c>
       <c r="F7" s="15" t="inlineStr">
         <is>
-          <t>Delivery</t>
+          <t>Bo Berg</t>
         </is>
       </c>
       <c r="G7" s="15" t="inlineStr">
         <is>
-          <t>Bo Berg</t>
-        </is>
-      </c>
-      <c r="H7" s="15" t="inlineStr">
-        <is>
           <t>Arctic Link</t>
-        </is>
-      </c>
-      <c r="I7" s="16" t="inlineStr">
-        <is>
-          <t>Amber</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="11" t="inlineStr">
         <is>
-          <t>Weather hold</t>
+          <t>Scope workshop</t>
         </is>
       </c>
       <c r="B8" s="14" t="n">
-        <v>46244</v>
+        <v>46214</v>
       </c>
       <c r="C8" s="14" t="n">
-        <v>46252</v>
-      </c>
-      <c r="D8" s="11" t="n"/>
-      <c r="E8" s="13" t="n">
-        <v>0</v>
+        <v>46228</v>
+      </c>
+      <c r="D8" s="13" t="n">
+        <v>50</v>
+      </c>
+      <c r="E8" s="11" t="inlineStr">
+        <is>
+          <t>Initiation</t>
+        </is>
       </c>
       <c r="F8" s="11" t="inlineStr">
         <is>
-          <t>Delivery</t>
+          <t>Cara Diaz</t>
         </is>
       </c>
       <c r="G8" s="11" t="inlineStr">
         <is>
-          <t>Riley Chen</t>
-        </is>
-      </c>
-      <c r="H8" s="11" t="inlineStr">
-        <is>
-          <t>Arctic Link</t>
-        </is>
-      </c>
-      <c r="I8" s="19" t="inlineStr">
-        <is>
-          <t>Red</t>
+          <t>Yard Retrofit</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="15" t="inlineStr">
         <is>
-          <t>On-call week</t>
+          <t>Scope freeze</t>
         </is>
       </c>
       <c r="B9" s="18" t="n">
-        <v>46252</v>
+        <v>46246</v>
       </c>
       <c r="C9" s="18" t="n">
-        <v>46258</v>
-      </c>
-      <c r="D9" s="15" t="n"/>
-      <c r="E9" s="17" t="n">
+        <v>46246</v>
+      </c>
+      <c r="D9" s="17" t="n">
         <v>0</v>
       </c>
+      <c r="E9" s="15" t="inlineStr">
+        <is>
+          <t>Initiation</t>
+        </is>
+      </c>
       <c r="F9" s="15" t="inlineStr">
         <is>
-          <t>Delivery</t>
+          <t>Cara Diaz</t>
         </is>
       </c>
       <c r="G9" s="15" t="inlineStr">
         <is>
-          <t>Bo Berg</t>
-        </is>
-      </c>
-      <c r="H9" s="15" t="inlineStr">
-        <is>
-          <t>Arctic Link</t>
-        </is>
-      </c>
-      <c r="I9" s="19" t="inlineStr">
-        <is>
-          <t>Red</t>
+          <t>Yard Retrofit</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="11" t="inlineStr">
         <is>
-          <t>Scope workshop</t>
+          <t>Integration</t>
         </is>
       </c>
       <c r="B10" s="14" t="n">
-        <v>46214</v>
+        <v>46204</v>
       </c>
       <c r="C10" s="14" t="n">
-        <v>46228</v>
-      </c>
-      <c r="D10" s="11" t="n"/>
-      <c r="E10" s="13" t="n">
-        <v>50</v>
+        <v>46244</v>
+      </c>
+      <c r="D10" s="13" t="n">
+        <v>85</v>
+      </c>
+      <c r="E10" s="11" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
       </c>
       <c r="F10" s="11" t="inlineStr">
         <is>
-          <t>Initiation</t>
+          <t>Sam Ortiz</t>
         </is>
       </c>
       <c r="G10" s="11" t="inlineStr">
         <is>
-          <t>Cara Diaz</t>
-        </is>
-      </c>
-      <c r="H10" s="11" t="inlineStr">
-        <is>
-          <t>Yard Retrofit</t>
-        </is>
-      </c>
-      <c r="I10" s="16" t="inlineStr">
-        <is>
-          <t>Amber</t>
+          <t>Digital Twin v2</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="15" t="inlineStr">
         <is>
-          <t>Budget review</t>
+          <t>UAT</t>
         </is>
       </c>
       <c r="B11" s="18" t="n">
-        <v>46223</v>
+        <v>46245</v>
       </c>
       <c r="C11" s="18" t="n">
-        <v>46239</v>
-      </c>
-      <c r="D11" s="15" t="n"/>
-      <c r="E11" s="17" t="n">
-        <v>15</v>
+        <v>46259</v>
+      </c>
+      <c r="D11" s="17" t="n">
+        <v>30</v>
+      </c>
+      <c r="E11" s="15" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
       </c>
       <c r="F11" s="15" t="inlineStr">
         <is>
-          <t>Initiation</t>
+          <t>Ada Ng</t>
         </is>
       </c>
       <c r="G11" s="15" t="inlineStr">
         <is>
-          <t>Finn Olsen</t>
-        </is>
-      </c>
-      <c r="H11" s="15" t="inlineStr">
-        <is>
-          <t>Yard Retrofit</t>
-        </is>
-      </c>
-      <c r="I11" s="19" t="inlineStr">
-        <is>
-          <t>Red</t>
+          <t>Digital Twin v2</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="11" t="inlineStr">
         <is>
-          <t>Scope freeze</t>
+          <t>Permit draft</t>
         </is>
       </c>
       <c r="B12" s="14" t="n">
-        <v>46246</v>
+        <v>46249</v>
       </c>
       <c r="C12" s="14" t="n">
-        <v>46246</v>
-      </c>
-      <c r="D12" s="11" t="n"/>
-      <c r="E12" s="13" t="n">
-        <v>0</v>
+        <v>46296</v>
+      </c>
+      <c r="D12" s="13" t="n">
+        <v>10</v>
+      </c>
+      <c r="E12" s="11" t="inlineStr">
+        <is>
+          <t>Plan</t>
+        </is>
       </c>
       <c r="F12" s="11" t="inlineStr">
         <is>
-          <t>Initiation</t>
+          <t>Finn Olsen</t>
         </is>
       </c>
       <c r="G12" s="11" t="inlineStr">
         <is>
-          <t>Cara Diaz</t>
-        </is>
-      </c>
-      <c r="H12" s="11" t="inlineStr">
-        <is>
-          <t>Yard Retrofit</t>
-        </is>
-      </c>
-      <c r="I12" s="19" t="inlineStr">
-        <is>
-          <t>Red</t>
+          <t>Port Expansion</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="15" t="inlineStr">
         <is>
-          <t>Model training</t>
+          <t>Stakeholder map</t>
         </is>
       </c>
       <c r="B13" s="18" t="n">
-        <v>46124</v>
+        <v>46254</v>
       </c>
       <c r="C13" s="18" t="n">
-        <v>46203</v>
-      </c>
-      <c r="D13" s="15" t="n"/>
-      <c r="E13" s="17" t="n">
-        <v>100</v>
+        <v>46280</v>
+      </c>
+      <c r="D13" s="17" t="n">
+        <v>5</v>
+      </c>
+      <c r="E13" s="15" t="inlineStr">
+        <is>
+          <t>Plan</t>
+        </is>
       </c>
       <c r="F13" s="15" t="inlineStr">
         <is>
-          <t>Build</t>
+          <t>Jordan Lee</t>
         </is>
       </c>
       <c r="G13" s="15" t="inlineStr">
         <is>
-          <t>Dan Okonkwo</t>
-        </is>
-      </c>
-      <c r="H13" s="15" t="inlineStr">
-        <is>
-          <t>Digital Twin v2</t>
-        </is>
-      </c>
-      <c r="I13" s="12" t="inlineStr">
-        <is>
-          <t>Green</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="11" t="inlineStr">
-        <is>
-          <t>Integration</t>
-        </is>
-      </c>
-      <c r="B14" s="14" t="n">
-        <v>46204</v>
-      </c>
-      <c r="C14" s="14" t="n">
-        <v>46244</v>
-      </c>
-      <c r="D14" s="11" t="n"/>
-      <c r="E14" s="13" t="n">
-        <v>85</v>
-      </c>
-      <c r="F14" s="11" t="inlineStr">
-        <is>
-          <t>Build</t>
-        </is>
-      </c>
-      <c r="G14" s="11" t="inlineStr">
-        <is>
-          <t>Sam Ortiz</t>
-        </is>
-      </c>
-      <c r="H14" s="11" t="inlineStr">
-        <is>
-          <t>Digital Twin v2</t>
-        </is>
-      </c>
-      <c r="I14" s="12" t="inlineStr">
-        <is>
-          <t>Green</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="15" t="inlineStr">
-        <is>
-          <t>UAT</t>
-        </is>
-      </c>
-      <c r="B15" s="18" t="n">
-        <v>46245</v>
-      </c>
-      <c r="C15" s="18" t="n">
-        <v>46259</v>
-      </c>
-      <c r="D15" s="15" t="n"/>
-      <c r="E15" s="17" t="n">
-        <v>30</v>
-      </c>
-      <c r="F15" s="15" t="inlineStr">
-        <is>
-          <t>Build</t>
-        </is>
-      </c>
-      <c r="G15" s="15" t="inlineStr">
-        <is>
-          <t>Ada Ng</t>
-        </is>
-      </c>
-      <c r="H15" s="15" t="inlineStr">
-        <is>
-          <t>Digital Twin v2</t>
-        </is>
-      </c>
-      <c r="I15" s="16" t="inlineStr">
-        <is>
-          <t>Amber</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="11" t="inlineStr">
-        <is>
-          <t>QA soak</t>
-        </is>
-      </c>
-      <c r="B16" s="14" t="n">
-        <v>46254</v>
-      </c>
-      <c r="C16" s="11" t="n"/>
-      <c r="D16" s="11" t="n">
-        <v>14</v>
-      </c>
-      <c r="E16" s="13" t="n">
-        <v>10</v>
-      </c>
-      <c r="F16" s="11" t="inlineStr">
-        <is>
-          <t>Build</t>
-        </is>
-      </c>
-      <c r="G16" s="11" t="inlineStr">
-        <is>
-          <t>Riley Chen</t>
-        </is>
-      </c>
-      <c r="H16" s="11" t="inlineStr">
-        <is>
-          <t>Digital Twin v2</t>
-        </is>
-      </c>
-      <c r="I16" s="12" t="inlineStr">
-        <is>
-          <t>Green</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="15" t="inlineStr">
-        <is>
-          <t>Permit draft</t>
-        </is>
-      </c>
-      <c r="B17" s="18" t="n">
-        <v>46249</v>
-      </c>
-      <c r="C17" s="18" t="n">
-        <v>46296</v>
-      </c>
-      <c r="D17" s="15" t="n"/>
-      <c r="E17" s="17" t="n">
-        <v>10</v>
-      </c>
-      <c r="F17" s="15" t="inlineStr">
-        <is>
-          <t>Plan</t>
-        </is>
-      </c>
-      <c r="G17" s="15" t="inlineStr">
-        <is>
-          <t>Finn Olsen</t>
-        </is>
-      </c>
-      <c r="H17" s="15" t="inlineStr">
-        <is>
           <t>Port Expansion</t>
         </is>
       </c>
-      <c r="I17" s="16" t="inlineStr">
-        <is>
-          <t>Amber</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="11" t="inlineStr">
-        <is>
-          <t>Stakeholder map</t>
-        </is>
-      </c>
-      <c r="B18" s="14" t="n">
-        <v>46254</v>
-      </c>
-      <c r="C18" s="14" t="n">
-        <v>46280</v>
-      </c>
-      <c r="D18" s="11" t="n"/>
-      <c r="E18" s="13" t="n">
-        <v>5</v>
-      </c>
-      <c r="F18" s="11" t="inlineStr">
-        <is>
-          <t>Plan</t>
-        </is>
-      </c>
-      <c r="G18" s="11" t="inlineStr">
-        <is>
-          <t>Jordan Lee</t>
-        </is>
-      </c>
-      <c r="H18" s="11" t="inlineStr">
-        <is>
-          <t>Port Expansion</t>
-        </is>
-      </c>
-      <c r="I18" s="12" t="inlineStr">
-        <is>
-          <t>Green</t>
-        </is>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I18"/>
+  <autoFilter ref="A1:G13"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Simplify suite starter to one grain per attribute
Drop Group from Projects so PMs are not maintaining the same phase
twice; document Project-as-link vs Project lead vs Resource clearly
on Start here to prevent wrong well bindings.

Co-authored-by: JonasL <Prez0@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/public/downloads/DatalundSuiteSample.xlsx
+++ b/public/downloads/DatalundSuiteSample.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Tasks" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Projects'!$A$1:$G$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Projects'!$A$1:$F$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Tasks'!$A$1:$G$13</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -559,10 +559,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="88" customWidth="1" min="1" max="1"/>
+    <col width="92" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
@@ -583,7 +583,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Seven columns. Replace the rows with your projects and tasks.</t>
+          <t>Two grains — portfolio vs assignments. Each attribute lives on one sheet.</t>
         </is>
       </c>
       <c r="B2" s="4" t="n"/>
@@ -615,7 +615,7 @@
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>3. Bind matching column names (see below)</t>
+          <t>3. Bind from the sheet that owns the column (see below)</t>
         </is>
       </c>
     </row>
@@ -623,56 +623,85 @@
     <row r="9" ht="20" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>What to maintain</t>
+          <t>What to maintain (no duplicates)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>Projects → DataLund Task List: Project, RAG, Group, Project lead, Progress, Start Date, End Date</t>
+          <t>Projects (Task List): Project · RAG · Project lead · Progress · Start Date · End Date</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>Tasks → Gantt + Resource Load: Task, Start Date, End Date, Progress, Group, Resource, Project</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="8" t="inlineStr">
-        <is>
-          <t>Progress is 0–100. RAG is Red / Amber / Green (or Rød / Gul / Grønn).</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="8" t="inlineStr">
-        <is>
-          <t>Same start and end date = milestone. Duration and Tooltips are optional later — not in this starter.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14"/>
+          <t>Tasks (Gantt + Resource Load): Task · Start Date · End Date · Progress · Group · Resource · Project</t>
+        </is>
+      </c>
+    </row>
+    <row r="12"/>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>How the sheets connect</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>Tasks[Project] is only the link to Projects — not a second project name to redesign.</t>
+        </is>
+      </c>
+    </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>Put Task List on the page, click a project — Gantt and Resource Load follow.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16"/>
+          <t>Project lead = who owns the project. Resource = who does the task. Different people, different wells.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>Group lives on Tasks (Gantt sections). Do not copy Group onto Projects in this starter.</t>
+        </is>
+      </c>
+    </row>
     <row r="17">
-      <c r="A17" s="9" t="inlineStr">
-        <is>
-          <t>https://datalund.no</t>
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>Gantt Resource well → Tasks[Resource]. Never put Project in the Resource well.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t>Progress is 0–100. RAG is Red / Amber / Green (or Rød / Gul / Grønn).</t>
+        </is>
+      </c>
+    </row>
+    <row r="19"/>
+    <row r="20">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>Put Task List on the page, click a project — Gantt and Resource Load follow.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21"/>
+    <row r="22">
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>https://datalund.no</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="8" t="inlineStr">
         <is>
           <t>Free Power BI visuals · support@datalund.no</t>
         </is>
@@ -684,7 +713,7 @@
     <mergeCell ref="A1:E1"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A17" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A22" r:id="rId1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -697,16 +726,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
@@ -722,25 +750,20 @@
       </c>
       <c r="C1" s="10" t="inlineStr">
         <is>
-          <t>Group</t>
+          <t>Project lead</t>
         </is>
       </c>
       <c r="D1" s="10" t="inlineStr">
         <is>
-          <t>Project lead</t>
+          <t>Progress</t>
         </is>
       </c>
       <c r="E1" s="10" t="inlineStr">
         <is>
-          <t>Progress</t>
+          <t>Start Date</t>
         </is>
       </c>
       <c r="F1" s="10" t="inlineStr">
-        <is>
-          <t>Start Date</t>
-        </is>
-      </c>
-      <c r="G1" s="10" t="inlineStr">
         <is>
           <t>End Date</t>
         </is>
@@ -759,21 +782,16 @@
       </c>
       <c r="C2" s="11" t="inlineStr">
         <is>
-          <t>Delivery</t>
-        </is>
-      </c>
-      <c r="D2" s="11" t="inlineStr">
-        <is>
           <t>Ada Ng</t>
         </is>
       </c>
-      <c r="E2" s="13" t="n">
+      <c r="D2" s="13" t="n">
         <v>72</v>
       </c>
+      <c r="E2" s="14" t="n">
+        <v>46184</v>
+      </c>
       <c r="F2" s="14" t="n">
-        <v>46184</v>
-      </c>
-      <c r="G2" s="14" t="n">
         <v>46284</v>
       </c>
     </row>
@@ -790,21 +808,16 @@
       </c>
       <c r="C3" s="15" t="inlineStr">
         <is>
-          <t>Delivery</t>
-        </is>
-      </c>
-      <c r="D3" s="15" t="inlineStr">
-        <is>
           <t>Bo Berg</t>
         </is>
       </c>
-      <c r="E3" s="17" t="n">
+      <c r="D3" s="17" t="n">
         <v>45</v>
       </c>
+      <c r="E3" s="18" t="n">
+        <v>46154</v>
+      </c>
       <c r="F3" s="18" t="n">
-        <v>46154</v>
-      </c>
-      <c r="G3" s="18" t="n">
         <v>46264</v>
       </c>
     </row>
@@ -821,21 +834,16 @@
       </c>
       <c r="C4" s="11" t="inlineStr">
         <is>
-          <t>Initiation</t>
-        </is>
-      </c>
-      <c r="D4" s="11" t="inlineStr">
-        <is>
           <t>Cara Diaz</t>
         </is>
       </c>
-      <c r="E4" s="13" t="n">
+      <c r="D4" s="13" t="n">
         <v>18</v>
       </c>
+      <c r="E4" s="14" t="n">
+        <v>46214</v>
+      </c>
       <c r="F4" s="14" t="n">
-        <v>46214</v>
-      </c>
-      <c r="G4" s="14" t="n">
         <v>46254</v>
       </c>
     </row>
@@ -852,21 +860,16 @@
       </c>
       <c r="C5" s="15" t="inlineStr">
         <is>
-          <t>Build</t>
-        </is>
-      </c>
-      <c r="D5" s="15" t="inlineStr">
-        <is>
           <t>Dan Okonkwo</t>
         </is>
       </c>
-      <c r="E5" s="17" t="n">
+      <c r="D5" s="17" t="n">
         <v>88</v>
       </c>
+      <c r="E5" s="18" t="n">
+        <v>46124</v>
+      </c>
       <c r="F5" s="18" t="n">
-        <v>46124</v>
-      </c>
-      <c r="G5" s="18" t="n">
         <v>46259</v>
       </c>
     </row>
@@ -883,26 +886,21 @@
       </c>
       <c r="C6" s="11" t="inlineStr">
         <is>
-          <t>Plan</t>
-        </is>
-      </c>
-      <c r="D6" s="11" t="inlineStr">
-        <is>
           <t>Finn Olsen</t>
         </is>
       </c>
-      <c r="E6" s="13" t="n">
+      <c r="D6" s="13" t="n">
         <v>12</v>
       </c>
+      <c r="E6" s="14" t="n">
+        <v>46249</v>
+      </c>
       <c r="F6" s="14" t="n">
-        <v>46249</v>
-      </c>
-      <c r="G6" s="14" t="n">
         <v>46424</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G6"/>
+  <autoFilter ref="A1:F6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Drop per-task Progress from suite starter
Keep RAG and Progress on Projects as portfolio health only. Tasks stay
schedule + Group + Resource + Project link so PMs are not updating
status at two grains.

Co-authored-by: JonasL <Prez0@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/public/downloads/DatalundSuiteSample.xlsx
+++ b/public/downloads/DatalundSuiteSample.xlsx
@@ -13,7 +13,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Projects'!$A$1:$F$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Tasks'!$A$1:$G$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Tasks'!$A$1:$F$13</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -559,7 +559,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="92" customWidth="1" min="1" max="1"/>
@@ -637,7 +637,7 @@
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>Tasks (Gantt + Resource Load): Task · Start Date · End Date · Progress · Group · Resource · Project</t>
+          <t>Tasks (Gantt + Resource Load): Task · Start Date · End Date · Group · Resource · Project</t>
         </is>
       </c>
     </row>
@@ -671,37 +671,44 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="8" t="inlineStr">
-        <is>
-          <t>Gantt Resource well → Tasks[Resource]. Never put Project in the Resource well.</t>
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>RAG + Progress on Projects is the portfolio health — not a second Progress on every task.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="8" t="inlineStr">
         <is>
-          <t>Progress is 0–100. RAG is Red / Amber / Green (or Rød / Gul / Grønn).</t>
-        </is>
-      </c>
-    </row>
-    <row r="19"/>
-    <row r="20">
-      <c r="A20" s="7" t="inlineStr">
+          <t>Gantt Resource well → Tasks[Resource]. Never put Project in the Resource well.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t>Task Progress is optional later for bar fill. Progress on Projects is 0–100. RAG: Red / Amber / Green.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20"/>
+    <row r="21">
+      <c r="A21" s="7" t="inlineStr">
         <is>
           <t>Put Task List on the page, click a project — Gantt and Resource Load follow.</t>
         </is>
       </c>
     </row>
-    <row r="21"/>
-    <row r="22">
-      <c r="A22" s="9" t="inlineStr">
+    <row r="22"/>
+    <row r="23">
+      <c r="A23" s="9" t="inlineStr">
         <is>
           <t>https://datalund.no</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="8" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="8" t="inlineStr">
         <is>
           <t>Free Power BI visuals · support@datalund.no</t>
         </is>
@@ -713,7 +720,7 @@
     <mergeCell ref="A1:E1"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A22" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A23" r:id="rId1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -912,7 +919,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -942,20 +949,15 @@
       </c>
       <c r="D1" s="10" t="inlineStr">
         <is>
-          <t>Progress</t>
+          <t>Group</t>
         </is>
       </c>
       <c r="E1" s="10" t="inlineStr">
         <is>
-          <t>Group</t>
+          <t>Resource</t>
         </is>
       </c>
       <c r="F1" s="10" t="inlineStr">
-        <is>
-          <t>Resource</t>
-        </is>
-      </c>
-      <c r="G1" s="10" t="inlineStr">
         <is>
           <t>Project</t>
         </is>
@@ -973,20 +975,17 @@
       <c r="C2" s="14" t="n">
         <v>46198</v>
       </c>
-      <c r="D2" s="13" t="n">
-        <v>100</v>
+      <c r="D2" s="11" t="inlineStr">
+        <is>
+          <t>Delivery</t>
+        </is>
       </c>
       <c r="E2" s="11" t="inlineStr">
         <is>
-          <t>Delivery</t>
+          <t>Ada Ng</t>
         </is>
       </c>
       <c r="F2" s="11" t="inlineStr">
-        <is>
-          <t>Ada Ng</t>
-        </is>
-      </c>
-      <c r="G2" s="11" t="inlineStr">
         <is>
           <t>North Sea Hub</t>
         </is>
@@ -1004,20 +1003,17 @@
       <c r="C3" s="18" t="n">
         <v>46223</v>
       </c>
-      <c r="D3" s="17" t="n">
-        <v>75</v>
+      <c r="D3" s="15" t="inlineStr">
+        <is>
+          <t>Delivery</t>
+        </is>
       </c>
       <c r="E3" s="15" t="inlineStr">
         <is>
-          <t>Delivery</t>
+          <t>Sam Ortiz</t>
         </is>
       </c>
       <c r="F3" s="15" t="inlineStr">
-        <is>
-          <t>Sam Ortiz</t>
-        </is>
-      </c>
-      <c r="G3" s="15" t="inlineStr">
         <is>
           <t>North Sea Hub</t>
         </is>
@@ -1035,20 +1031,17 @@
       <c r="C4" s="14" t="n">
         <v>46270</v>
       </c>
-      <c r="D4" s="13" t="n">
-        <v>20</v>
+      <c r="D4" s="11" t="inlineStr">
+        <is>
+          <t>Delivery</t>
+        </is>
       </c>
       <c r="E4" s="11" t="inlineStr">
         <is>
-          <t>Delivery</t>
+          <t>Ada Ng</t>
         </is>
       </c>
       <c r="F4" s="11" t="inlineStr">
-        <is>
-          <t>Ada Ng</t>
-        </is>
-      </c>
-      <c r="G4" s="11" t="inlineStr">
         <is>
           <t>North Sea Hub</t>
         </is>
@@ -1066,20 +1059,17 @@
       <c r="C5" s="18" t="n">
         <v>46254</v>
       </c>
-      <c r="D5" s="17" t="n">
-        <v>40</v>
+      <c r="D5" s="15" t="inlineStr">
+        <is>
+          <t>Delivery</t>
+        </is>
       </c>
       <c r="E5" s="15" t="inlineStr">
         <is>
-          <t>Delivery</t>
+          <t>Bo Berg</t>
         </is>
       </c>
       <c r="F5" s="15" t="inlineStr">
-        <is>
-          <t>Bo Berg</t>
-        </is>
-      </c>
-      <c r="G5" s="15" t="inlineStr">
         <is>
           <t>Arctic Link</t>
         </is>
@@ -1097,20 +1087,17 @@
       <c r="C6" s="14" t="n">
         <v>46252</v>
       </c>
-      <c r="D6" s="13" t="n">
-        <v>0</v>
+      <c r="D6" s="11" t="inlineStr">
+        <is>
+          <t>Delivery</t>
+        </is>
       </c>
       <c r="E6" s="11" t="inlineStr">
         <is>
-          <t>Delivery</t>
+          <t>Riley Chen</t>
         </is>
       </c>
       <c r="F6" s="11" t="inlineStr">
-        <is>
-          <t>Riley Chen</t>
-        </is>
-      </c>
-      <c r="G6" s="11" t="inlineStr">
         <is>
           <t>Arctic Link</t>
         </is>
@@ -1128,20 +1115,17 @@
       <c r="C7" s="18" t="n">
         <v>46258</v>
       </c>
-      <c r="D7" s="17" t="n">
-        <v>0</v>
+      <c r="D7" s="15" t="inlineStr">
+        <is>
+          <t>Delivery</t>
+        </is>
       </c>
       <c r="E7" s="15" t="inlineStr">
         <is>
-          <t>Delivery</t>
+          <t>Bo Berg</t>
         </is>
       </c>
       <c r="F7" s="15" t="inlineStr">
-        <is>
-          <t>Bo Berg</t>
-        </is>
-      </c>
-      <c r="G7" s="15" t="inlineStr">
         <is>
           <t>Arctic Link</t>
         </is>
@@ -1159,20 +1143,17 @@
       <c r="C8" s="14" t="n">
         <v>46228</v>
       </c>
-      <c r="D8" s="13" t="n">
-        <v>50</v>
+      <c r="D8" s="11" t="inlineStr">
+        <is>
+          <t>Initiation</t>
+        </is>
       </c>
       <c r="E8" s="11" t="inlineStr">
         <is>
-          <t>Initiation</t>
+          <t>Cara Diaz</t>
         </is>
       </c>
       <c r="F8" s="11" t="inlineStr">
-        <is>
-          <t>Cara Diaz</t>
-        </is>
-      </c>
-      <c r="G8" s="11" t="inlineStr">
         <is>
           <t>Yard Retrofit</t>
         </is>
@@ -1190,20 +1171,17 @@
       <c r="C9" s="18" t="n">
         <v>46246</v>
       </c>
-      <c r="D9" s="17" t="n">
-        <v>0</v>
+      <c r="D9" s="15" t="inlineStr">
+        <is>
+          <t>Initiation</t>
+        </is>
       </c>
       <c r="E9" s="15" t="inlineStr">
         <is>
-          <t>Initiation</t>
+          <t>Cara Diaz</t>
         </is>
       </c>
       <c r="F9" s="15" t="inlineStr">
-        <is>
-          <t>Cara Diaz</t>
-        </is>
-      </c>
-      <c r="G9" s="15" t="inlineStr">
         <is>
           <t>Yard Retrofit</t>
         </is>
@@ -1221,20 +1199,17 @@
       <c r="C10" s="14" t="n">
         <v>46244</v>
       </c>
-      <c r="D10" s="13" t="n">
-        <v>85</v>
+      <c r="D10" s="11" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
       </c>
       <c r="E10" s="11" t="inlineStr">
         <is>
-          <t>Build</t>
+          <t>Sam Ortiz</t>
         </is>
       </c>
       <c r="F10" s="11" t="inlineStr">
-        <is>
-          <t>Sam Ortiz</t>
-        </is>
-      </c>
-      <c r="G10" s="11" t="inlineStr">
         <is>
           <t>Digital Twin v2</t>
         </is>
@@ -1252,20 +1227,17 @@
       <c r="C11" s="18" t="n">
         <v>46259</v>
       </c>
-      <c r="D11" s="17" t="n">
-        <v>30</v>
+      <c r="D11" s="15" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
       </c>
       <c r="E11" s="15" t="inlineStr">
         <is>
-          <t>Build</t>
+          <t>Ada Ng</t>
         </is>
       </c>
       <c r="F11" s="15" t="inlineStr">
-        <is>
-          <t>Ada Ng</t>
-        </is>
-      </c>
-      <c r="G11" s="15" t="inlineStr">
         <is>
           <t>Digital Twin v2</t>
         </is>
@@ -1283,20 +1255,17 @@
       <c r="C12" s="14" t="n">
         <v>46296</v>
       </c>
-      <c r="D12" s="13" t="n">
-        <v>10</v>
+      <c r="D12" s="11" t="inlineStr">
+        <is>
+          <t>Plan</t>
+        </is>
       </c>
       <c r="E12" s="11" t="inlineStr">
         <is>
-          <t>Plan</t>
+          <t>Finn Olsen</t>
         </is>
       </c>
       <c r="F12" s="11" t="inlineStr">
-        <is>
-          <t>Finn Olsen</t>
-        </is>
-      </c>
-      <c r="G12" s="11" t="inlineStr">
         <is>
           <t>Port Expansion</t>
         </is>
@@ -1314,27 +1283,24 @@
       <c r="C13" s="18" t="n">
         <v>46280</v>
       </c>
-      <c r="D13" s="17" t="n">
-        <v>5</v>
+      <c r="D13" s="15" t="inlineStr">
+        <is>
+          <t>Plan</t>
+        </is>
       </c>
       <c r="E13" s="15" t="inlineStr">
         <is>
-          <t>Plan</t>
+          <t>Jordan Lee</t>
         </is>
       </c>
       <c r="F13" s="15" t="inlineStr">
         <is>
-          <t>Jordan Lee</t>
-        </is>
-      </c>
-      <c r="G13" s="15" t="inlineStr">
-        <is>
           <t>Port Expansion</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G13"/>
+  <autoFilter ref="A1:F13"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>